<commit_message>
feat: L0-02 Pipeline CI/CD et registre d'images privé
- Add multi-stage Dockerfiles for api, web, worker (node:24-alpine)
- Add .dockerignore files for each app
- Add docker-compose.yml for dev environment (postgres, api, web, worker, pgadmin)
- Add docker-compose.override.yml for hot reload development
- Add deploy-dev.sh script for automated dev deployment
- Update CI workflow with:
  - Security scans: npm audit, OSV scanner, Gitleaks
  - Build & push multi-arch images to GHCR with SemVer tagging
  - Trivy container scanning with SARIF upload
  - Automatic dev deployment on main branch push
- Add dependabot.yml for automated dependency updates
- Add AGPL-3.0-only LICENSE file
- Update all package.json files with AGPL-3.0-only license
- Add SPDX license headers to Dockerfiles
- Update ticket L0-02 status to Terminé
- Regenerate backlog artifacts and velocity
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -717,7 +717,7 @@
       <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr"/>
@@ -796,7 +796,7 @@
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: update backlog & velocity (tickets problem_json_filter, swagger_ui → Terminé)
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -3313,7 +3313,7 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr"/>
@@ -3469,7 +3469,7 @@
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: RFC 9457 error format + Swagger UI (L0-34, L0-36) (#9)
* docs: update backlog & velocity (tickets problem_json_filter, swagger_ui → Terminé)

* feat: RFC 9457 error format + Swagger UI (L0-34, L0-36)

- Add RequestIdMiddleware for x-request-id header and tracing
- Update ValidationPipe to output validationErrors with field names for RFC 9457 errors array
- Rewrite HttpExceptionFilter to ProblemJsonFilter with full RFC 9457 compliance
- Allow /api/docs* routes without authentication in JwtAuthGuard
- Add SwaggerModule setup at /api/docs with BearerAuth, tags, version
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -3313,7 +3313,7 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr"/>
@@ -3469,7 +3469,7 @@
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: add RBAC acceptance criteria to L1/L2 tickets depending on rbac
- L1-01 (annees): @Permissions('annee:read')/@Permissions('annee:write') on all controller routes; default deny (403)
- L1-07 (ens): @Permissions('enseignant:read')/@Permissions('enseignant:write') on all controller routes; default deny (403)
- L2-06 (repartitions): @Permissions on all routes; ScopeGuard returns 404 out of department
- L2-12 (validate): @Permissions('repartition:validate') on POST validate; ImmutabilityGuard applies even to Administrator

Signed-off-by: Cline
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -3593,7 +3593,8 @@
         <is>
           <t>- Unicité du code d'année et du couple (année, numéro)
 - Seul l'Administrateur écrit ; les autres rôles lisent
-- Un semestre compte 14 semaines par défaut</t>
+- Un semestre compte 14 semaines par défaut
+- Toutes les routes du contrôleur d'années sont protégées par @Permissions('annee:read')/@Permissions('annee:write') ; toute route non décorée est refusée par défaut (403)</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -4297,7 +4298,8 @@
         <is>
           <t>- Unicité (année, matricule)
 - Désactivation refusée (409) si présent dans une répartition d'une année non clôturée
-- Le Responsable modifie les modules enseignables de son département uniquement</t>
+- Le Responsable modifie les modules enseignables de son département uniquement
+- Toutes les routes du contrôleur enseignants sont protégées par @Permissions('enseignant:read')/@Permissions('enseignant:write') ; toute route non décorée est refusée par défaut (403)</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -6097,7 +6099,9 @@
       <c r="H71" s="5" t="inlineStr">
         <is>
           <t>- Création automatique à l'ouverture du semestre
-- Consultation par Administrateur, Gestionnaire, Direction (lecture) et Responsable</t>
+- Consultation par Administrateur, Gestionnaire, Direction (lecture) et Responsable
+- Toutes les routes du contrôleur de répartitions sont protégées par @Permissions('repartition:read')/@Permissions('repartition:write')/@Permissions('repartition:validate') ; toute route non décorée est refusée par défaut (403)
+- ScopeGuard renvoie 404 pour une répartition hors du département du Responsable (pas de révélation d'existence)</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
@@ -6569,7 +6573,9 @@
 - Création d'un snapshot immuable (affectations, tag résolu, charges, jeu de règles, hash)
 - Triggers append-only sur SnapshotAffectation et SnapshotCharge
 - SnapshotCharge conserve volume brut, charge calculée, charge de référence, décharges, service dû, écart, heures sup
-- Validation par l'Administrateur tracée (parAdministrateur) avec notification au Responsable (L5)</t>
+- Validation par l'Administrateur tracée (parAdministrateur) avec notification au Responsable (L5)
+- La route POST /repartitions/{id}/validate est protégée par @Permissions('repartition:validate') (Responsable de département ou Administrateur uniquement)
+- ImmutabilityGuard s'applique : une fois validé, le snapshot ne peut plus être modifié, y compris par l'Administrateur</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: OpenAPI 3.1 généré avec désactivation en production (L0-21) (#29)
* docs: ticket L0-20 passe en En cours

* feat: OpenAPI 3.1 généré avec désactivation en production (L0-21)

- Ajouter la configuration OpenAPI (enabled, path) dans app.config.ts
- Désactiver Swagger UI /api/docs en production (NODE_ENV=production)
- Forcer OpenAPI 3.1.0 sur le document généré par SwaggerModule
- Ajouter le fichier .env.example avec variables OPENAPI_ENABLED / OPENAPI_PATH
- Ajouter 4 tests unitaires pour app.config (openapi configuration)
- Mettre à jour le backlog et la vélocité (L0-21 → En cours)

* docs: update backlog & velocity (ticket L0-21 → Terminé)
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -2765,7 +2765,7 @@
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr"/>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: comptes terminé, L0-23 en En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1823,7 +1823,7 @@
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P16" s="5" t="inlineStr"/>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(l0-23): admin users screen (list, create, toggle, form) (#32)
* docs: comptes terminé, L0-23 en En cours

* feat(l0-23): écran admin utilisateurs (liste, création, toggle, formulaire)

- Ajouter la page /admin/users avec liste, filtres, toggle actif, pagination
- Ajouter le dialog création/édition utilisateur (react-hook-form + zod)
- Ajouter l'API client (apiFetch, users, erreurs typées)
- Ajouter les hooks React Query (useUsers, useCreateUser, useUpdateUser, etc.)
- Ajouter le composant Toast (sonner) et l'intégrer au layout
- Ajouter les messages i18n français
- Corriger la résolution des modules @takt/contracts vers dist

* docs: backlog & velocity (ticket L0-23 admin_ui → Terminé)
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1823,7 +1823,7 @@
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P16" s="5" t="inlineStr"/>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: correct L0 ticket coherence (duplicate IDs, statuses, backlog regeneration)
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr"/>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: mark ticket L1-01 (annees) as En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Epics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$211</definedName>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P41" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: set L0-39 to L0-42 to En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -2059,7 +2059,7 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P19" s="5" t="inlineStr"/>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P23" s="5" t="inlineStr"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P26" s="5" t="inlineStr"/>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: mark L0-39 to L0-42 as Terminé and regenerate backlog & velocity
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -2059,7 +2059,7 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P19" s="5" t="inlineStr"/>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P23" s="5" t="inlineStr"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P26" s="5" t="inlineStr"/>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: regenerate backlog artifacts after L0 closure
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr"/>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P15" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: add backlog tickets L7-18 (ordre + dnd-kit) and L7-19 (frontend tests)
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$211</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P211"/>
+  <dimension ref="A1:P213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -17104,8 +17104,168 @@
       </c>
       <c r="P211" s="5" t="inlineStr"/>
     </row>
+    <row r="212">
+      <c r="A212" s="5" t="inlineStr">
+        <is>
+          <t>L7-18</t>
+        </is>
+      </c>
+      <c r="B212" s="5" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="C212" s="5" t="inlineStr">
+        <is>
+          <t>E7.6</t>
+        </is>
+      </c>
+      <c r="D212" s="5" t="inlineStr">
+        <is>
+          <t>Arborescence de structure</t>
+        </is>
+      </c>
+      <c r="E212" s="5" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="F212" s="5" t="inlineStr">
+        <is>
+          <t>Champ ordre et réordonnancement dnd-kit de l'arbre de structure</t>
+        </is>
+      </c>
+      <c r="G212" s="5" t="inlineStr">
+        <is>
+          <t>Ajouter le champ ordre aux modèles Departement, Formation, Niveau, Groupe ; endpoints de réordonnancement backend ; intégration dnd-kit dans StructureTree avec optimistic UI et rollback ; tri par ordre puis code.</t>
+        </is>
+      </c>
+      <c r="H212" s="5" t="inlineStr">
+        <is>
+          <t>- Ajout du champ ordre Int @default(0) aux 4 modèles Prisma avec index sur (branche, ordre)
+- Endpoints PATCH /departements/reorder, /formations/reorder, /niveaux/reorder, /groupes/reorder
+- Intégration DndContext + useSortable dans structure-tree.tsx
+- Optimistic UI avec rollback en cas d'erreur 4xx
+- Messages i18n en français</t>
+        </is>
+      </c>
+      <c r="I212" s="5" t="inlineStr">
+        <is>
+          <t>EX-ORG-01, EX-ORG-02</t>
+        </is>
+      </c>
+      <c r="J212" s="5" t="inlineStr">
+        <is>
+          <t>§3.3</t>
+        </is>
+      </c>
+      <c r="K212" s="5" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="L212" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="M212" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N212" s="5" t="inlineStr">
+        <is>
+          <t>L1-09</t>
+        </is>
+      </c>
+      <c r="O212" s="5" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="P212" s="5" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="5" t="inlineStr">
+        <is>
+          <t>L7-19</t>
+        </is>
+      </c>
+      <c r="B213" s="5" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="C213" s="5" t="inlineStr">
+        <is>
+          <t>E7.7</t>
+        </is>
+      </c>
+      <c r="D213" s="5" t="inlineStr">
+        <is>
+          <t>Qualité frontend</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="F213" s="5" t="inlineStr">
+        <is>
+          <t>Tests frontend (Zod, API, hooks, composant StructureTree)</t>
+        </is>
+      </c>
+      <c r="G213" s="5" t="inlineStr">
+        <is>
+          <t>Ajouter vitest, testing-library, jsdom ; écrire des tests unitaires pour la validation Zod, les fonctions API, les hooks React Query et le composant StructureTree.</t>
+        </is>
+      </c>
+      <c r="H213" s="5" t="inlineStr">
+        <is>
+          <t>- Configuration vitest.config.ts avec jsdom et alias @/
+- Tests de validation Zod pour structure.ts
+- Tests des fonctions API (lib/api/structure.ts)
+- Tests des hooks (use-structure.ts)
+- Tests du composant StructureTree</t>
+        </is>
+      </c>
+      <c r="I213" s="5" t="inlineStr">
+        <is>
+          <t>EX-NFR-07</t>
+        </is>
+      </c>
+      <c r="J213" s="5" t="inlineStr">
+        <is>
+          <t>§5.5</t>
+        </is>
+      </c>
+      <c r="K213" s="5" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="L213" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="M213" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="N213" s="5" t="inlineStr">
+        <is>
+          <t>L1-09, L7-18</t>
+        </is>
+      </c>
+      <c r="O213" s="5" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="P213" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P211"/>
+  <autoFilter ref="A1:P213"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17165,15 +17325,15 @@
         </is>
       </c>
       <c r="C2" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A2)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A2)</f>
         <v/>
       </c>
       <c r="D2" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A2,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A2,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E2" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A2,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A2,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17189,15 +17349,15 @@
         </is>
       </c>
       <c r="C3" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A3)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A3)</f>
         <v/>
       </c>
       <c r="D3" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A3,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A3,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E3" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A3,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A3,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17213,15 +17373,15 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A4)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A4)</f>
         <v/>
       </c>
       <c r="D4" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A4,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A4,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E4" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A4,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A4,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17237,15 +17397,15 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A5)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A5)</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A5,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A5,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A5,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A5,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17261,15 +17421,15 @@
         </is>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A6)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A6)</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A6,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A6,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A6,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A6,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17285,15 +17445,15 @@
         </is>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A7)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A7)</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A7,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A7,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A7,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A7,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17309,15 +17469,15 @@
         </is>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A8)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A8)</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A8,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A8,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E8" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A8,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A8,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17333,15 +17493,15 @@
         </is>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIF(Tickets!$B$2:$B$211,A9)</f>
+        <f>COUNTIF(Tickets!$B$2:$B$213,A9)</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>SUMIF(Tickets!$B$2:$B$211,A9,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$B$2:$B$213,A9,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
       <c r="E9" s="5">
-        <f>SUMIFS(Tickets!$M$2:$M$211,Tickets!$B$2:$B$211,A9,Tickets!$O$2:$O$211,"Terminé")</f>
+        <f>SUMIFS(Tickets!$M$2:$M$213,Tickets!$B$2:$B$213,A9,Tickets!$O$2:$O$213,"Terminé")</f>
         <v/>
       </c>
     </row>
@@ -17375,7 +17535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -17429,11 +17589,11 @@
         </is>
       </c>
       <c r="D2" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A2)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A2)</f>
         <v/>
       </c>
       <c r="E2" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A2,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A2,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17454,11 +17614,11 @@
         </is>
       </c>
       <c r="D3" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A3)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A3)</f>
         <v/>
       </c>
       <c r="E3" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A3,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A3,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17479,11 +17639,11 @@
         </is>
       </c>
       <c r="D4" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A4)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A4)</f>
         <v/>
       </c>
       <c r="E4" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A4,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A4,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17504,11 +17664,11 @@
         </is>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A5)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A5)</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A5,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A5,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17529,11 +17689,11 @@
         </is>
       </c>
       <c r="D6" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A6)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A6)</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A6,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A6,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17554,11 +17714,11 @@
         </is>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A7)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A7)</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A7,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A7,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17579,11 +17739,11 @@
         </is>
       </c>
       <c r="D8" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A8)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A8)</f>
         <v/>
       </c>
       <c r="E8" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A8,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A8,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17604,11 +17764,11 @@
         </is>
       </c>
       <c r="D9" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A9)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A9)</f>
         <v/>
       </c>
       <c r="E9" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A9,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A9,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17629,11 +17789,11 @@
         </is>
       </c>
       <c r="D10" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A10)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A10)</f>
         <v/>
       </c>
       <c r="E10" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A10,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A10,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17654,11 +17814,11 @@
         </is>
       </c>
       <c r="D11" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A11)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A11)</f>
         <v/>
       </c>
       <c r="E11" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A11,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A11,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17679,11 +17839,11 @@
         </is>
       </c>
       <c r="D12" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A12)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A12)</f>
         <v/>
       </c>
       <c r="E12" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A12,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A12,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17704,11 +17864,11 @@
         </is>
       </c>
       <c r="D13" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A13)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A13)</f>
         <v/>
       </c>
       <c r="E13" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A13,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A13,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17729,11 +17889,11 @@
         </is>
       </c>
       <c r="D14" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A14)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A14)</f>
         <v/>
       </c>
       <c r="E14" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A14,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A14,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17754,11 +17914,11 @@
         </is>
       </c>
       <c r="D15" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A15)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A15)</f>
         <v/>
       </c>
       <c r="E15" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A15,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A15,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17779,11 +17939,11 @@
         </is>
       </c>
       <c r="D16" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A16)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A16)</f>
         <v/>
       </c>
       <c r="E16" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A16,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A16,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17804,11 +17964,11 @@
         </is>
       </c>
       <c r="D17" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A17)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A17)</f>
         <v/>
       </c>
       <c r="E17" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A17,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A17,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17829,11 +17989,11 @@
         </is>
       </c>
       <c r="D18" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A18)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A18)</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A18,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A18,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17854,11 +18014,11 @@
         </is>
       </c>
       <c r="D19" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A19)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A19)</f>
         <v/>
       </c>
       <c r="E19" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A19,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A19,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17879,11 +18039,11 @@
         </is>
       </c>
       <c r="D20" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A20)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A20)</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A20,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A20,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17904,11 +18064,11 @@
         </is>
       </c>
       <c r="D21" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A21)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A21)</f>
         <v/>
       </c>
       <c r="E21" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A21,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A21,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17929,11 +18089,11 @@
         </is>
       </c>
       <c r="D22" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A22)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A22)</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A22,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A22,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17954,11 +18114,11 @@
         </is>
       </c>
       <c r="D23" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A23)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A23)</f>
         <v/>
       </c>
       <c r="E23" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A23,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A23,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -17979,11 +18139,11 @@
         </is>
       </c>
       <c r="D24" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A24)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A24)</f>
         <v/>
       </c>
       <c r="E24" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A24,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A24,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18004,11 +18164,11 @@
         </is>
       </c>
       <c r="D25" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A25)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A25)</f>
         <v/>
       </c>
       <c r="E25" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A25,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A25,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18029,11 +18189,11 @@
         </is>
       </c>
       <c r="D26" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A26)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A26)</f>
         <v/>
       </c>
       <c r="E26" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A26,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A26,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18054,11 +18214,11 @@
         </is>
       </c>
       <c r="D27" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A27)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A27)</f>
         <v/>
       </c>
       <c r="E27" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A27,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A27,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18079,11 +18239,11 @@
         </is>
       </c>
       <c r="D28" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A28)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A28)</f>
         <v/>
       </c>
       <c r="E28" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A28,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A28,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18104,11 +18264,11 @@
         </is>
       </c>
       <c r="D29" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A29)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A29)</f>
         <v/>
       </c>
       <c r="E29" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A29,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A29,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18129,11 +18289,11 @@
         </is>
       </c>
       <c r="D30" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A30)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A30)</f>
         <v/>
       </c>
       <c r="E30" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A30,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A30,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18154,11 +18314,11 @@
         </is>
       </c>
       <c r="D31" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A31)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A31)</f>
         <v/>
       </c>
       <c r="E31" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A31,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A31,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18179,11 +18339,11 @@
         </is>
       </c>
       <c r="D32" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A32)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A32)</f>
         <v/>
       </c>
       <c r="E32" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A32,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A32,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18204,11 +18364,11 @@
         </is>
       </c>
       <c r="D33" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A33)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A33)</f>
         <v/>
       </c>
       <c r="E33" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A33,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A33,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18229,11 +18389,11 @@
         </is>
       </c>
       <c r="D34" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A34)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A34)</f>
         <v/>
       </c>
       <c r="E34" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A34,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A34,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18254,11 +18414,11 @@
         </is>
       </c>
       <c r="D35" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A35)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A35)</f>
         <v/>
       </c>
       <c r="E35" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A35,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A35,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18279,11 +18439,11 @@
         </is>
       </c>
       <c r="D36" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A36)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A36)</f>
         <v/>
       </c>
       <c r="E36" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A36,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A36,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18304,11 +18464,11 @@
         </is>
       </c>
       <c r="D37" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A37)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A37)</f>
         <v/>
       </c>
       <c r="E37" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A37,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A37,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18329,11 +18489,11 @@
         </is>
       </c>
       <c r="D38" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A38)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A38)</f>
         <v/>
       </c>
       <c r="E38" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A38,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A38,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18354,11 +18514,11 @@
         </is>
       </c>
       <c r="D39" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A39)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A39)</f>
         <v/>
       </c>
       <c r="E39" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A39,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A39,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18379,11 +18539,11 @@
         </is>
       </c>
       <c r="D40" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A40)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A40)</f>
         <v/>
       </c>
       <c r="E40" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A40,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A40,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18404,11 +18564,11 @@
         </is>
       </c>
       <c r="D41" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A41)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A41)</f>
         <v/>
       </c>
       <c r="E41" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A41,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A41,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18429,11 +18589,11 @@
         </is>
       </c>
       <c r="D42" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A42)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A42)</f>
         <v/>
       </c>
       <c r="E42" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A42,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A42,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18454,11 +18614,11 @@
         </is>
       </c>
       <c r="D43" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A43)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A43)</f>
         <v/>
       </c>
       <c r="E43" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A43,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A43,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18479,11 +18639,11 @@
         </is>
       </c>
       <c r="D44" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A44)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A44)</f>
         <v/>
       </c>
       <c r="E44" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A44,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A44,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18504,11 +18664,11 @@
         </is>
       </c>
       <c r="D45" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A45)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A45)</f>
         <v/>
       </c>
       <c r="E45" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A45,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A45,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18529,11 +18689,11 @@
         </is>
       </c>
       <c r="D46" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A46)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A46)</f>
         <v/>
       </c>
       <c r="E46" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A46,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A46,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18554,11 +18714,11 @@
         </is>
       </c>
       <c r="D47" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A47)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A47)</f>
         <v/>
       </c>
       <c r="E47" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A47,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A47,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18579,11 +18739,11 @@
         </is>
       </c>
       <c r="D48" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A48)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A48)</f>
         <v/>
       </c>
       <c r="E48" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A48,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A48,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18604,11 +18764,11 @@
         </is>
       </c>
       <c r="D49" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A49)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A49)</f>
         <v/>
       </c>
       <c r="E49" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A49,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A49,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18629,11 +18789,11 @@
         </is>
       </c>
       <c r="D50" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A50)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A50)</f>
         <v/>
       </c>
       <c r="E50" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A50,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A50,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18654,11 +18814,11 @@
         </is>
       </c>
       <c r="D51" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A51)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A51)</f>
         <v/>
       </c>
       <c r="E51" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A51,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A51,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18679,11 +18839,11 @@
         </is>
       </c>
       <c r="D52" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A52)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A52)</f>
         <v/>
       </c>
       <c r="E52" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A52,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A52,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18704,11 +18864,11 @@
         </is>
       </c>
       <c r="D53" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A53)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A53)</f>
         <v/>
       </c>
       <c r="E53" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A53,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A53,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18729,11 +18889,11 @@
         </is>
       </c>
       <c r="D54" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A54)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A54)</f>
         <v/>
       </c>
       <c r="E54" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A54,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A54,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18754,11 +18914,11 @@
         </is>
       </c>
       <c r="D55" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A55)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A55)</f>
         <v/>
       </c>
       <c r="E55" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A55,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A55,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18779,11 +18939,11 @@
         </is>
       </c>
       <c r="D56" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A56)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A56)</f>
         <v/>
       </c>
       <c r="E56" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A56,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A56,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18804,11 +18964,11 @@
         </is>
       </c>
       <c r="D57" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A57)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A57)</f>
         <v/>
       </c>
       <c r="E57" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A57,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A57,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18829,11 +18989,11 @@
         </is>
       </c>
       <c r="D58" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A58)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A58)</f>
         <v/>
       </c>
       <c r="E58" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A58,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A58,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18854,11 +19014,11 @@
         </is>
       </c>
       <c r="D59" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A59)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A59)</f>
         <v/>
       </c>
       <c r="E59" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A59,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A59,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18879,11 +19039,11 @@
         </is>
       </c>
       <c r="D60" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A60)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A60)</f>
         <v/>
       </c>
       <c r="E60" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A60,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A60,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
@@ -18904,26 +19064,76 @@
         </is>
       </c>
       <c r="D61" s="7">
-        <f>COUNTIF(Tickets!$C$2:$C$211,A61)</f>
+        <f>COUNTIF(Tickets!$C$2:$C$213,A61)</f>
         <v/>
       </c>
       <c r="E61" s="7">
-        <f>SUMIF(Tickets!$C$2:$C$211,A61,Tickets!$M$2:$M$211)</f>
+        <f>SUMIF(Tickets!$C$2:$C$213,A61,Tickets!$M$2:$M$213)</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>E7.6</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Arborescence de structure</t>
+        </is>
+      </c>
+      <c r="D62" s="7">
+        <f>COUNTIF(Tickets!$C$2:$C$213,A62)</f>
+        <v/>
+      </c>
+      <c r="E62" s="7">
+        <f>SUMIF(Tickets!$C$2:$C$213,A62,Tickets!$M$2:$M$213)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>E7.7</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Qualité frontend</t>
+        </is>
+      </c>
+      <c r="D63" s="7">
+        <f>COUNTIF(Tickets!$C$2:$C$213,A63)</f>
+        <v/>
+      </c>
+      <c r="E63" s="7">
+        <f>SUMIF(Tickets!$C$2:$C$213,A63,Tickets!$M$2:$M$213)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D62" s="3">
-        <f>SUM(D2:D61)</f>
+      <c r="D64" s="3">
+        <f>SUM(D2:D63)</f>
         <v/>
       </c>
-      <c r="E62" s="3">
-        <f>SUM(E2:E61)</f>
+      <c r="E64" s="3">
+        <f>SUM(E2:E63)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark tickets L7-18 and L7-19 as Terminé
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -17179,7 +17179,7 @@
       </c>
       <c r="O212" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P212" s="5" t="inlineStr"/>
@@ -17259,7 +17259,7 @@
       </c>
       <c r="O213" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P213" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: passer L1-18 Generateur grille horaire a En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -4954,7 +4954,7 @@
       </c>
       <c r="O56" s="5" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P56" s="5" t="inlineStr"/>
@@ -5113,7 +5113,7 @@
       </c>
       <c r="O58" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P58" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: mark L3-01 En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$213</definedName>
@@ -7391,7 +7391,7 @@
       </c>
       <c r="O87" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P87" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: mark L2-01 En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$219</definedName>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="O74" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P74" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: corriger statuts backlog après audit de cohérence git
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Epics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$219</definedName>
@@ -717,7 +717,7 @@
       <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr"/>
@@ -953,7 +953,7 @@
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr"/>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr"/>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr"/>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P19" s="5" t="inlineStr"/>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P21" s="5" t="inlineStr"/>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P23" s="5" t="inlineStr"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P24" s="5" t="inlineStr"/>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P25" s="5" t="inlineStr"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P26" s="5" t="inlineStr"/>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P27" s="5" t="inlineStr"/>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr"/>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr"/>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P30" s="5" t="inlineStr"/>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr"/>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr"/>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr"/>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr"/>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P36" s="5" t="inlineStr"/>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr"/>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P39" s="5" t="inlineStr"/>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P53" s="5" t="inlineStr"/>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P55" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: corriger statuts backlog après vérification code (22 tickets L0-L3 déjà implémentés)
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -953,7 +953,7 @@
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr"/>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P19" s="5" t="inlineStr"/>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P23" s="5" t="inlineStr"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P24" s="5" t="inlineStr"/>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P25" s="5" t="inlineStr"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P26" s="5" t="inlineStr"/>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr"/>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr"/>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr"/>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr"/>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P53" s="5" t="inlineStr"/>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P55" s="5" t="inlineStr"/>
@@ -17029,7 +17029,7 @@
       </c>
       <c r="O210" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P210" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: marquer 9 tickets Terminé et régénérer artefacts backlog
L0-20 rbac_test, L0-32 jwt_guard, L0-33 roles_guard, L0-34 users_module,
L0-35 problem_json_filter, L0-36 link_header, L0-38 security_event,
L1-13 salles, L1-15 compat : implémentation déjà présente dans le code,
passage de À faire à Terminé.

Régénération des artefacts : tickets_data.py, Backlog_TAKT_tickets.csv,
Backlog_TAKT.xlsx, VELOCITE.md (59 tickets terminés au total).
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$219</definedName>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P21" s="5" t="inlineStr"/>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr"/>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr"/>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr"/>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P36" s="5" t="inlineStr"/>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr"/>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P39" s="5" t="inlineStr"/>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P53" s="5" t="inlineStr"/>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P55" s="5" t="inlineStr"/>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="O75" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P75" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: mark L0-01, L0-05, L0-06, L0-26, L0-27, L0-28 as Terminé; revert L7-10 backup to À faire
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -717,7 +717,7 @@
       <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr"/>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr"/>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr"/>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P27" s="5" t="inlineStr"/>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr"/>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr"/>
@@ -17029,7 +17029,7 @@
       </c>
       <c r="O210" s="5" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="P210" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: mark det-imp-01 En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Epics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$219</definedName>
@@ -5898,7 +5898,7 @@
       </c>
       <c r="O68" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P68" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: mark L2-03 En cours
</commit_message>
<xml_diff>
--- a/docs/Backlog_TAKT.xlsx
+++ b/docs/Backlog_TAKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tickets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Epics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$P$219</definedName>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="O76" s="5" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="P76" s="5" t="inlineStr"/>

</xml_diff>